<commit_message>
feat: Enhance USD transaction detection in BBVA Mastercard parsing to resolve classification errors and improve accuracy
</commit_message>
<xml_diff>
--- a/output/BBVA_MASTERCARD_20250315.xlsx
+++ b/output/BBVA_MASTERCARD_20250315.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,16 +463,18 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Onlyfans.Com</t>
+          <t>SU PAGO EN PESOS</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>35</v>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>-123695,0</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -483,23 +485,187 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2025-07-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Platzi 557227</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>15725,0</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>BBVA Mastercard</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>2025-03-15</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>ON FIT</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ON FIT C.05/06 006805</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
         <is>
           <t>ARS</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>107970</v>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>107970,0</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>BBVA Mastercard</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-07-07</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Onlyfans.Com USD 35,00</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>35,0</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>BBVA Mastercard</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-07-25</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MERPAGO*FUARK C.01/03 421094</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>69152,68</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>BBVA Mastercard</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-07-31</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>IIBB PERCEP-CABA 2,00%( 46025,00)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>920,5</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BBVA Mastercard</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2025-07-31</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>IVA RG 4240 21%( 46025,00)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>9665,25</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BBVA Mastercard</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2025-07-31</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DB.RG 5617 30% ( 46025,00 )</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ARS</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>13807,5</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>BBVA Mastercard</t>
         </is>

</xml_diff>